<commit_message>
Sync data dictionaries from public_api_docs
</commit_message>
<xml_diff>
--- a/data_dictionaries/en/Belvo_Data_Dictionary_en.xlsx
+++ b/data_dictionaries/en/Belvo_Data_Dictionary_en.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -873,14 +873,18 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>form_fields</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr"/>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>This field is **deprecated** and will be removed in a future release. Please use the `id` field instead, which is the unique identifier for the institution.</t>
+        </is>
+      </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -891,7 +895,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -900,22 +904,14 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].name</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>The username, password, or username type field.</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>username</t>
-        </is>
-      </c>
+          <t>form_fields</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>array</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -935,17 +931,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].type</t>
+          <t>form_fields[].name</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>The input type for the form field. For example, string.</t>
+          <t>The username, password, or username type field.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>username</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -970,10 +966,45 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>form_fields[].type</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>The input type for the form field. For example, string.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>form_fields[].label</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The label of the form field. For example:
 - Client number
@@ -982,44 +1013,9 @@
 </t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Client number</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>form_fields[].validation</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>The type of input validation used for the field.</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>^.{1,}$</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1044,17 +1040,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].placeholder</t>
+          <t>form_fields[].validation</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>The placeholder text in the form field.</t>
+          <t>The type of input validation used for the field.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>ABC333333A33</t>
+          <t>^.{1,}$</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1079,17 +1075,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].validation_message</t>
+          <t>form_fields[].placeholder</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>The message displayed when an invalid input is provided in the form field.</t>
+          <t>The placeholder text in the form field.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Invalid client number</t>
+          <t>ABC333333A33</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1114,55 +1110,55 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>form_fields[].validation_message</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>The message displayed when an invalid input is provided in the form field.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Invalid client number</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>form_fields[].values</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">If the form field is for documents, the institution may require additional
 input regarding the document type.
 </t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>array</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>form_fields[].values[].code</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>The code of the document.</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -1182,10 +1178,45 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>form_fields[].values[].code</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>The code of the document.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>form_fields[].values[].label</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The label for the field. For example:
 - Cédula de Ciudadanía
@@ -1194,44 +1225,9 @@
 </t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Cédula de Ciudadanía</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>form_fields[].values[].validation</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>The type of input validation used for the field.</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>^.{1,}$</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1256,17 +1252,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].values[].validation_message</t>
+          <t>form_fields[].values[].validation</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>The message displayed when an invalid input is provided in the form field.</t>
+          <t>The type of input validation used for the field.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Invalid document number</t>
+          <t>^.{1,}$</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1291,17 +1287,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].values[].placeholder</t>
+          <t>form_fields[].values[].validation_message</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>The placeholder text in the form field.</t>
+          <t>The message displayed when an invalid input is provided in the form field.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>DEF4444908M22</t>
+          <t>Invalid document number</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1326,10 +1322,45 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>form_fields[].values[].placeholder</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>The placeholder text in the form field.</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>DEF4444908M22</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>features</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The features that the institution supports. If the institution has no special features, then Belvo returns an empty array.
 Here is a list of the available features:
@@ -1337,45 +1368,10 @@
 </t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>array</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>features[].name</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>The name of the feature.</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>token_required</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
@@ -1395,17 +1391,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>features[].description</t>
+          <t>features[].name</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>The description of the feature.</t>
+          <t>The name of the feature.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>The institution may require a token during link creation or login</t>
+          <t>token_required</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1430,10 +1426,45 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>features[].description</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>The description of the feature.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>The institution may require a token during link creation or login</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>resources</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">A list of Belvo resources that you can use with the institution. This list includes one or more of the following resources:
   - `ACCOUNTS`
@@ -1457,37 +1488,37 @@
 </t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>["ACCOUNTS", "BALANCES", "INCOMES", "OWNERS", "RECURRING_EXPENSES", "RISK_INSIGHTS", "TRANSACTIONS"]</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>array</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>integration_type</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The type of technology used to access the institution. We return one of the following values:
 - `credentials`: Uses Belvo's scraping technology, combined with user credentials, to perform requests.
@@ -1495,49 +1526,9 @@
 </t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>credentials</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>credentials, openfinance</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Indicates whether Belvo's integration with the institution is currently active (`healthy`) or undergoing maintenance (`down`).
-</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>healthy</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1558,7 +1549,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>healthy, down</t>
+          <t>credentials, openfinance</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1566,18 +1557,23 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>openbanking_information</t>
+          <t>status</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Information about the institution on the Open Finance environment.</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
+          <t xml:space="preserve">Indicates whether Belvo's integration with the institution is currently active (`healthy`) or undergoing maintenance (`down`).
+</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
@@ -1588,31 +1584,31 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>healthy, down</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>openbanking_information.description</t>
+          <t>openbanking_information</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>A short description of the institution on the Open Finance environment. Extracted from Open Finance regulated institutions listing.</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>A 1ss Bank é uma fintech fundada em janeiro de 2020, com a missão de ajudar empresas com grandes ecossistemas a se tornarem fintechs, integrando e automatizando seus processos financeiros através de APIs e plataforma white-label.</t>
-        </is>
-      </c>
+          <t>Information about the institution on the Open Finance environment.</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>object</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
@@ -1632,22 +1628,22 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>openbanking_information.participants</t>
+          <t>openbanking_information.description</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>List of brands' servers available from the institution in Open Finance. Extracted from Open Finance regulated institutions listing.</t>
+          <t>A short description of the institution on the Open Finance environment. Extracted from Open Finance regulated institutions listing.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>["1ss Bank"]</t>
+          <t>A 1ss Bank é uma fintech fundada em janeiro de 2020, com a missão de ajudar empresas com grandes ecossistemas a se tornarem fintechs, integrando e automatizando seus processos financeiros através de APIs e plataforma white-label.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
@@ -1667,29 +1663,25 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>openbanking_information.authorization_server_id</t>
+          <t>openbanking_information.participants</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>The authorization server ID (UUID) of the institution on the Open Finance Environment.</t>
+          <t>List of brands' servers available from the institution in Open Finance. Extracted from Open Finance regulated institutions listing.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>aa18fcd3-2f0b-40b1-87db-8930b10b78b1</t>
+          <t>["1ss Bank"]</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -1702,6 +1694,45 @@
       </c>
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>openbanking_information.authorization_server_id</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>The authorization server ID (UUID) of the institution on the Open Finance Environment.</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>aa18fcd3-2f0b-40b1-87db-8930b10b78b1</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -48441,7 +48472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -48657,17 +48688,18 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>expired_at</t>
+          <t>institution_display_name</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The ISO-8601 timestamp when the consent will expire. In the case that `undefined_consent_expiration` is `true`, this field will be `null`.</t>
+          <t xml:space="preserve">The display name of the banking institution that the consent is related to.
+</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2021-02-27T13:01:41.941Z</t>
+          <t>Mock Bank</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -48675,11 +48707,7 @@
           <t>string</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>date-time</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -48696,22 +48724,23 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>undefined_consent_expiration</t>
+          <t>institution_icon_logo</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Indicated whether the consent is for an undefined period, that is, that there is no expiration for the consent.</t>
+          <t xml:space="preserve">The URL to the banking institution's logo.
+</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>https://assets.belvo.io/institutions/mockbank/logo.svg</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -48731,18 +48760,18 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>belvo_organization_name</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ISO-8601 timestamp of when the data point was created in Belvo's database.
+          <t xml:space="preserve">The name registered in Belvo of the organization that created the link.
 </t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2022-02-09T08:45:50.406032Z</t>
+          <t>ACME Corporation</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -48750,11 +48779,7 @@
           <t>string</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>date-time</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -48771,10 +48796,241 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>link_id</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Belvo link ID that the consent belongs to.
+</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2e5d2c5e-6b3a-4b5c-8d1e-9f0a1b2c3d4e</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>user_name</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The name provided in `consent.identification_info.name` during the initial Widget Access Token Request.
+</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Jack White</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>expired_at</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>The ISO-8601 timestamp when the consent will expire. In the case that `undefined_consent_expiration` is `true`, this field will be `null`.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2021-02-27T13:01:41.941Z</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>date-time</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>undefined_consent_expiration</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Indicated whether the consent is for an undefined period, that is, that there is no expiration for the consent.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>consent_duration</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The duration of the consent in days. In the case that `undefined_consent_expiration` is `true`, this field will be `null`.
+Possible values:
+- `92` (3 months)
+- `183` (6 months)
+- `275` (9 months)
+- `366` (12 months)
+</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>366</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The ISO-8601 timestamp of when the data point was created in Belvo's database.
+</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2022-02-09T08:45:50.406032Z</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>date-time</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The status of the consent in the open finance network. Can be either:
   - `AUTHORISED`: The consent is still valid for use until the `expired_at` date.
@@ -48786,224 +49042,14 @@
 </t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>AUTHORISED</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>AUTHORISED, AWAITING_AUTHORISATION_CONFIRMATION, AWAITING_AUTHORISATION, REJECTED, EXPIRED, None</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>permissions</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Details regarding the permissions attached to the consent.</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>permissions.ACCOUNTS</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>A list of of open banking permissions relating to accessing account information.</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>["ACCOUNTS_OVERDRAFT_LIMITS_READ", "ACCOUNTS_READ", "ACCOUNTS_TRANSACTIONS_READ", "ACCOUNTS_BALANCES_READ"]</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>permissions.CREDIT_CARDS</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>A list of of open banking permissions relating to accessing credit card information.</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>["CREDIT_CARDS_ACCOUNTS_LIMITS_READ", "CREDIT_CARDS_ACCOUNTS_BILLS_READ", "CREDIT_CARDS_ACCOUNTS_TRANSACTIONS_READ", "CREDIT_CARDS_ACCOUNTS_BILLS_TRANSACTIONS_READ", "CREDIT_CARDS_ACCOUNTS_READ"]</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>permissions.CREDIT_OPERATIONS</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>A list of of open banking permissions relating to accessing credit product information.</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>["LOANS_READ", "LOANS_WARRANTIES_READ", "LOANS_SCHEDULED_INSTALMENTS_READ", "LOANS_PAYMENTS_READ", "FINANCINGS_READ", "FINANCINGS_WARRANTIES_READ", "FINANCINGS_SCHEDULED_INSTALMENTS_READ", "FINANCINGS_PAYMENTS_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_WARRANTIES_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_SCHEDULED_INSTALMENTS_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_PAYMENTS_READ", "INVOICE_FINANCINGS_READ", "INVOICE_FINANCINGS_WARRANTIES_READ", "INVOICE_FINANCINGS_SCHEDULED_INSTALMENTS_READ", "INVOICE_FINANCINGS_PAYMENTS_READ"]</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>permissions.REGISTER</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>A list of of open banking permissions relating to accessing personal information.</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>["CUSTOMERS_PERSONAL_IDENTIFICATIONS_READ", "CUSTOMERS_PERSONAL_ADITTIONALINFO_READ"]</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>permissions.RESOURCES</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>A list of functional permissions required to interact with the permissions.</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>["RESOURCES_READ"]</t>
-        </is>
-      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -49014,11 +49060,256 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>AUTHORISED, AWAITING_AUTHORISATION_CONFIRMATION, AWAITING_AUTHORISATION, REJECTED, EXPIRED, None</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>permissions</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Details regarding the permissions attached to the consent.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>permissions.ACCOUNTS</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>A list of of open banking permissions relating to accessing account information.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>["ACCOUNTS_OVERDRAFT_LIMITS_READ", "ACCOUNTS_READ", "ACCOUNTS_TRANSACTIONS_READ", "ACCOUNTS_BALANCES_READ"]</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>permissions.CREDIT_CARDS</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>A list of of open banking permissions relating to accessing credit card information.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>["CREDIT_CARDS_ACCOUNTS_LIMITS_READ", "CREDIT_CARDS_ACCOUNTS_BILLS_READ", "CREDIT_CARDS_ACCOUNTS_TRANSACTIONS_READ", "CREDIT_CARDS_ACCOUNTS_BILLS_TRANSACTIONS_READ", "CREDIT_CARDS_ACCOUNTS_READ"]</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>permissions.CREDIT_OPERATIONS</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>A list of of open banking permissions relating to accessing credit product information.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>["LOANS_READ", "LOANS_WARRANTIES_READ", "LOANS_SCHEDULED_INSTALMENTS_READ", "LOANS_PAYMENTS_READ", "FINANCINGS_READ", "FINANCINGS_WARRANTIES_READ", "FINANCINGS_SCHEDULED_INSTALMENTS_READ", "FINANCINGS_PAYMENTS_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_WARRANTIES_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_SCHEDULED_INSTALMENTS_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_PAYMENTS_READ", "INVOICE_FINANCINGS_READ", "INVOICE_FINANCINGS_WARRANTIES_READ", "INVOICE_FINANCINGS_SCHEDULED_INSTALMENTS_READ", "INVOICE_FINANCINGS_PAYMENTS_READ"]</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>permissions.REGISTER</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>A list of of open banking permissions relating to accessing personal information.</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>["CUSTOMERS_PERSONAL_IDENTIFICATIONS_READ", "CUSTOMERS_PERSONAL_ADITTIONALINFO_READ"]</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>permissions.RESOURCES</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>A list of functional permissions required to interact with the permissions.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>["RESOURCES_READ"]</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>permissions.INVESTMENTS</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>A list of open banking permissions relating to accessing investment information.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>["BANK_FIXED_INCOMES_READ", "CREDIT_FIXED_INCOMES_READ", "FUNDS_READ", "VARIABLE_INCOMES_READ", "TREASURE_TITLES_READ"]</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sync data dictionaries from public_api_docs (#49)
Co-authored-by: github-actions[bot] <github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data_dictionaries/en/Belvo_Data_Dictionary_en.xlsx
+++ b/data_dictionaries/en/Belvo_Data_Dictionary_en.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -873,14 +873,18 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>form_fields</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr"/>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>This field is **deprecated** and will be removed in a future release. Please use the `id` field instead, which is the unique identifier for the institution.</t>
+        </is>
+      </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -891,7 +895,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -900,22 +904,14 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].name</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>The username, password, or username type field.</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>username</t>
-        </is>
-      </c>
+          <t>form_fields</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>array</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -935,17 +931,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].type</t>
+          <t>form_fields[].name</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>The input type for the form field. For example, string.</t>
+          <t>The username, password, or username type field.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>username</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -970,10 +966,45 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>form_fields[].type</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>The input type for the form field. For example, string.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>form_fields[].label</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The label of the form field. For example:
 - Client number
@@ -982,44 +1013,9 @@
 </t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Client number</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>form_fields[].validation</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>The type of input validation used for the field.</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>^.{1,}$</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1044,17 +1040,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].placeholder</t>
+          <t>form_fields[].validation</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>The placeholder text in the form field.</t>
+          <t>The type of input validation used for the field.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>ABC333333A33</t>
+          <t>^.{1,}$</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1079,17 +1075,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].validation_message</t>
+          <t>form_fields[].placeholder</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>The message displayed when an invalid input is provided in the form field.</t>
+          <t>The placeholder text in the form field.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Invalid client number</t>
+          <t>ABC333333A33</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1114,55 +1110,55 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>form_fields[].validation_message</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>The message displayed when an invalid input is provided in the form field.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Invalid client number</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>form_fields[].values</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">If the form field is for documents, the institution may require additional
 input regarding the document type.
 </t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>array</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>form_fields[].values[].code</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>The code of the document.</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -1182,10 +1178,45 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>form_fields[].values[].code</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>The code of the document.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>form_fields[].values[].label</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The label for the field. For example:
 - Cédula de Ciudadanía
@@ -1194,44 +1225,9 @@
 </t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Cédula de Ciudadanía</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>form_fields[].values[].validation</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>The type of input validation used for the field.</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>^.{1,}$</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1256,17 +1252,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].values[].validation_message</t>
+          <t>form_fields[].values[].validation</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>The message displayed when an invalid input is provided in the form field.</t>
+          <t>The type of input validation used for the field.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Invalid document number</t>
+          <t>^.{1,}$</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1291,17 +1287,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>form_fields[].values[].placeholder</t>
+          <t>form_fields[].values[].validation_message</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>The placeholder text in the form field.</t>
+          <t>The message displayed when an invalid input is provided in the form field.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>DEF4444908M22</t>
+          <t>Invalid document number</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1326,10 +1322,45 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>form_fields[].values[].placeholder</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>The placeholder text in the form field.</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>DEF4444908M22</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>features</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The features that the institution supports. If the institution has no special features, then Belvo returns an empty array.
 Here is a list of the available features:
@@ -1337,45 +1368,10 @@
 </t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>array</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>features[].name</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>The name of the feature.</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>token_required</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
@@ -1395,17 +1391,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>features[].description</t>
+          <t>features[].name</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>The description of the feature.</t>
+          <t>The name of the feature.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>The institution may require a token during link creation or login</t>
+          <t>token_required</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1430,10 +1426,45 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>features[].description</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>The description of the feature.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>The institution may require a token during link creation or login</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>resources</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">A list of Belvo resources that you can use with the institution. This list includes one or more of the following resources:
   - `ACCOUNTS`
@@ -1457,37 +1488,37 @@
 </t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>["ACCOUNTS", "BALANCES", "INCOMES", "OWNERS", "RECURRING_EXPENSES", "RISK_INSIGHTS", "TRANSACTIONS"]</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>array</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>integration_type</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The type of technology used to access the institution. We return one of the following values:
 - `credentials`: Uses Belvo's scraping technology, combined with user credentials, to perform requests.
@@ -1495,49 +1526,9 @@
 </t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>credentials</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>credentials, openfinance</t>
-        </is>
-      </c>
-      <c r="I29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Indicates whether Belvo's integration with the institution is currently active (`healthy`) or undergoing maintenance (`down`).
-</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>healthy</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1558,7 +1549,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>healthy, down</t>
+          <t>credentials, openfinance</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1566,18 +1557,23 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>openbanking_information</t>
+          <t>status</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Information about the institution on the Open Finance environment.</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
+          <t xml:space="preserve">Indicates whether Belvo's integration with the institution is currently active (`healthy`) or undergoing maintenance (`down`).
+</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
@@ -1588,31 +1584,31 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>healthy, down</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>openbanking_information.description</t>
+          <t>openbanking_information</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>A short description of the institution on the Open Finance environment. Extracted from Open Finance regulated institutions listing.</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>A 1ss Bank é uma fintech fundada em janeiro de 2020, com a missão de ajudar empresas com grandes ecossistemas a se tornarem fintechs, integrando e automatizando seus processos financeiros através de APIs e plataforma white-label.</t>
-        </is>
-      </c>
+          <t>Information about the institution on the Open Finance environment.</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>object</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
@@ -1632,22 +1628,22 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>openbanking_information.participants</t>
+          <t>openbanking_information.description</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>List of brands' servers available from the institution in Open Finance. Extracted from Open Finance regulated institutions listing.</t>
+          <t>A short description of the institution on the Open Finance environment. Extracted from Open Finance regulated institutions listing.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>["1ss Bank"]</t>
+          <t>A 1ss Bank é uma fintech fundada em janeiro de 2020, com a missão de ajudar empresas com grandes ecossistemas a se tornarem fintechs, integrando e automatizando seus processos financeiros através de APIs e plataforma white-label.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
@@ -1667,29 +1663,25 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>openbanking_information.authorization_server_id</t>
+          <t>openbanking_information.participants</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>The authorization server ID (UUID) of the institution on the Open Finance Environment.</t>
+          <t>List of brands' servers available from the institution in Open Finance. Extracted from Open Finance regulated institutions listing.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>aa18fcd3-2f0b-40b1-87db-8930b10b78b1</t>
+          <t>["1ss Bank"]</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -1702,6 +1694,45 @@
       </c>
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>openbanking_information.authorization_server_id</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>The authorization server ID (UUID) of the institution on the Open Finance Environment.</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>aa18fcd3-2f0b-40b1-87db-8930b10b78b1</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -48441,7 +48472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -48657,17 +48688,18 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>expired_at</t>
+          <t>institution_display_name</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The ISO-8601 timestamp when the consent will expire. In the case that `undefined_consent_expiration` is `true`, this field will be `null`.</t>
+          <t xml:space="preserve">The display name of the banking institution that the consent is related to.
+</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2021-02-27T13:01:41.941Z</t>
+          <t>Mock Bank</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -48675,11 +48707,7 @@
           <t>string</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>date-time</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -48696,22 +48724,23 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>undefined_consent_expiration</t>
+          <t>institution_icon_logo</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Indicated whether the consent is for an undefined period, that is, that there is no expiration for the consent.</t>
+          <t xml:space="preserve">The URL to the banking institution's logo.
+</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>https://assets.belvo.io/institutions/mockbank/logo.svg</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -48731,18 +48760,18 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>belvo_organization_name</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The ISO-8601 timestamp of when the data point was created in Belvo's database.
+          <t xml:space="preserve">The name registered in Belvo of the organization that created the link.
 </t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2022-02-09T08:45:50.406032Z</t>
+          <t>ACME Corporation</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -48750,11 +48779,7 @@
           <t>string</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>date-time</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -48771,10 +48796,241 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>link_id</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Belvo link ID that the consent belongs to.
+</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>2e5d2c5e-6b3a-4b5c-8d1e-9f0a1b2c3d4e</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>uuid</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>user_name</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The name provided in `consent.identification_info.name` during the initial Widget Access Token Request.
+</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Jack White</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>expired_at</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>The ISO-8601 timestamp when the consent will expire. In the case that `undefined_consent_expiration` is `true`, this field will be `null`.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2021-02-27T13:01:41.941Z</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>date-time</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>undefined_consent_expiration</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Indicated whether the consent is for an undefined period, that is, that there is no expiration for the consent.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>consent_duration</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The duration of the consent in days. In the case that `undefined_consent_expiration` is `true`, this field will be `null`.
+Possible values:
+- `92` (3 months)
+- `183` (6 months)
+- `275` (9 months)
+- `366` (12 months)
+</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>366</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The ISO-8601 timestamp of when the data point was created in Belvo's database.
+</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2022-02-09T08:45:50.406032Z</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>date-time</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The status of the consent in the open finance network. Can be either:
   - `AUTHORISED`: The consent is still valid for use until the `expired_at` date.
@@ -48786,224 +49042,14 @@
 </t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>AUTHORISED</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>AUTHORISED, AWAITING_AUTHORISATION_CONFIRMATION, AWAITING_AUTHORISATION, REJECTED, EXPIRED, None</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>permissions</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Details regarding the permissions attached to the consent.</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>permissions.ACCOUNTS</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>A list of of open banking permissions relating to accessing account information.</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>["ACCOUNTS_OVERDRAFT_LIMITS_READ", "ACCOUNTS_READ", "ACCOUNTS_TRANSACTIONS_READ", "ACCOUNTS_BALANCES_READ"]</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>permissions.CREDIT_CARDS</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>A list of of open banking permissions relating to accessing credit card information.</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>["CREDIT_CARDS_ACCOUNTS_LIMITS_READ", "CREDIT_CARDS_ACCOUNTS_BILLS_READ", "CREDIT_CARDS_ACCOUNTS_TRANSACTIONS_READ", "CREDIT_CARDS_ACCOUNTS_BILLS_TRANSACTIONS_READ", "CREDIT_CARDS_ACCOUNTS_READ"]</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>permissions.CREDIT_OPERATIONS</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>A list of of open banking permissions relating to accessing credit product information.</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>["LOANS_READ", "LOANS_WARRANTIES_READ", "LOANS_SCHEDULED_INSTALMENTS_READ", "LOANS_PAYMENTS_READ", "FINANCINGS_READ", "FINANCINGS_WARRANTIES_READ", "FINANCINGS_SCHEDULED_INSTALMENTS_READ", "FINANCINGS_PAYMENTS_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_WARRANTIES_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_SCHEDULED_INSTALMENTS_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_PAYMENTS_READ", "INVOICE_FINANCINGS_READ", "INVOICE_FINANCINGS_WARRANTIES_READ", "INVOICE_FINANCINGS_SCHEDULED_INSTALMENTS_READ", "INVOICE_FINANCINGS_PAYMENTS_READ"]</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>permissions.REGISTER</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>A list of of open banking permissions relating to accessing personal information.</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>["CUSTOMERS_PERSONAL_IDENTIFICATIONS_READ", "CUSTOMERS_PERSONAL_ADITTIONALINFO_READ"]</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>permissions.RESOURCES</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>A list of functional permissions required to interact with the permissions.</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>["RESOURCES_READ"]</t>
-        </is>
-      </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -49014,11 +49060,256 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>AUTHORISED, AWAITING_AUTHORISATION_CONFIRMATION, AWAITING_AUTHORISATION, REJECTED, EXPIRED, None</t>
+        </is>
+      </c>
       <c r="I15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>permissions</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Details regarding the permissions attached to the consent.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>permissions.ACCOUNTS</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>A list of of open banking permissions relating to accessing account information.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>["ACCOUNTS_OVERDRAFT_LIMITS_READ", "ACCOUNTS_READ", "ACCOUNTS_TRANSACTIONS_READ", "ACCOUNTS_BALANCES_READ"]</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>permissions.CREDIT_CARDS</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>A list of of open banking permissions relating to accessing credit card information.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>["CREDIT_CARDS_ACCOUNTS_LIMITS_READ", "CREDIT_CARDS_ACCOUNTS_BILLS_READ", "CREDIT_CARDS_ACCOUNTS_TRANSACTIONS_READ", "CREDIT_CARDS_ACCOUNTS_BILLS_TRANSACTIONS_READ", "CREDIT_CARDS_ACCOUNTS_READ"]</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>permissions.CREDIT_OPERATIONS</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>A list of of open banking permissions relating to accessing credit product information.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>["LOANS_READ", "LOANS_WARRANTIES_READ", "LOANS_SCHEDULED_INSTALMENTS_READ", "LOANS_PAYMENTS_READ", "FINANCINGS_READ", "FINANCINGS_WARRANTIES_READ", "FINANCINGS_SCHEDULED_INSTALMENTS_READ", "FINANCINGS_PAYMENTS_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_WARRANTIES_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_SCHEDULED_INSTALMENTS_READ", "UNARRANGED_ACCOUNTS_OVERDRAFT_PAYMENTS_READ", "INVOICE_FINANCINGS_READ", "INVOICE_FINANCINGS_WARRANTIES_READ", "INVOICE_FINANCINGS_SCHEDULED_INSTALMENTS_READ", "INVOICE_FINANCINGS_PAYMENTS_READ"]</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>permissions.REGISTER</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>A list of of open banking permissions relating to accessing personal information.</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>["CUSTOMERS_PERSONAL_IDENTIFICATIONS_READ", "CUSTOMERS_PERSONAL_ADITTIONALINFO_READ"]</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>permissions.RESOURCES</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>A list of functional permissions required to interact with the permissions.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>["RESOURCES_READ"]</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>permissions.INVESTMENTS</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>A list of open banking permissions relating to accessing investment information.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>["BANK_FIXED_INCOMES_READ", "CREDIT_FIXED_INCOMES_READ", "FUNDS_READ", "VARIABLE_INCOMES_READ", "TREASURE_TITLES_READ"]</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sync data dictionaries from public_api_docs (#51)
Co-authored-by: github-actions[bot] <github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data_dictionaries/en/Belvo_Data_Dictionary_en.xlsx
+++ b/data_dictionaries/en/Belvo_Data_Dictionary_en.xlsx
@@ -11435,7 +11435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -11697,22 +11697,22 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>internal_identification</t>
+          <t>days_since_extraction</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Unique ID for user according to the institution. For IMSS and ISSSTE Mexico, this is the CURP.</t>
+          <t>The number of days that have passed since the employment data was originally extracted from the institution.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>BLPM951331IONVGR54</t>
+          <t>42</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -11732,18 +11732,22 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>personal_data</t>
+          <t>internal_identification</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Details regarding the personal information of the individual.</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr"/>
+          <t>Unique ID for user according to the institution. For IMSS and ISSSTE Mexico, this is the CURP.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>BLPM951331IONVGR54</t>
+        </is>
+      </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -11763,23 +11767,18 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>personal_data.official_name</t>
+          <t>personal_data</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The legal name of the individual.
-</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Bruce Banner del Torro</t>
-        </is>
-      </c>
+          <t>Details regarding the personal information of the individual.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>object</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -11790,7 +11789,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -11799,18 +11798,18 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>personal_data.first_name</t>
+          <t>personal_data.official_name</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The first name of the individual.
+          <t xml:space="preserve">The legal name of the individual.
 </t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Bruce</t>
+          <t>Bruce Banner del Torro</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -11835,18 +11834,18 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>personal_data.last_name</t>
+          <t>personal_data.first_name</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The last name of the individual.
+          <t xml:space="preserve">The first name of the individual.
 </t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Banner del Torro</t>
+          <t>Bruce</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -11871,18 +11870,18 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>personal_data.birth_date</t>
+          <t>personal_data.last_name</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The date of birth of the individual, in `YYYY-MM-DD` format.
+          <t xml:space="preserve">The last name of the individual.
 </t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2022-02-09</t>
+          <t>Banner del Torro</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -11890,11 +11889,7 @@
           <t>string</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
+      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -11911,21 +11906,30 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>personal_data.entitlements</t>
+          <t>personal_data.birth_date</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Details regarding the benefits the individual is entitled to.</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
+          <t xml:space="preserve">The date of birth of the individual, in `YYYY-MM-DD` format.
+</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2022-02-09</t>
+        </is>
+      </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -11933,7 +11937,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -11942,23 +11946,18 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>personal_data.entitlements.entitled_to_health_insurance</t>
+          <t>personal_data.entitlements</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indicates whether or not the individual is entitled to health insurance.
-</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
+          <t>Details regarding the benefits the individual is entitled to.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>object</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
@@ -11978,12 +11977,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>personal_data.entitlements.entitled_to_company_benefits</t>
+          <t>personal_data.entitlements.entitled_to_health_insurance</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indicates whether or not the individual is entitled to company benefits.
+          <t xml:space="preserve">Indicates whether or not the individual is entitled to health insurance.
 </t>
         </is>
       </c>
@@ -12014,26 +12013,26 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>personal_data.entitlements.valid_until</t>
+          <t>personal_data.entitlements.entitled_to_company_benefits</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Date until when the individual is covered by health insurance and/or company benefits. If `null` the employee is currently working and no end date is required.
-</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
+          <t xml:space="preserve">Indicates whether or not the individual is entitled to company benefits.
+</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -12041,7 +12040,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -12050,10 +12049,46 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>personal_data.entitlements.valid_until</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date until when the individual is covered by health insurance and/or company benefits. If `null` the employee is currently working and no end date is required.
+</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>personal_data.entitlements.status</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Indicates the employment status of the individual. We return one of the following responses:
   - `EMPLOYED`
@@ -12063,49 +12098,14 @@
 </t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>EMPLOYED</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>EMPLOYED, RETIRED, UNEMPLOYED, null</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>personal_data.document_ids</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Details regarding the individual's ID documents.</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
@@ -12119,16 +12119,51 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>EMPLOYED, RETIRED, UNEMPLOYED, null</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>personal_data.document_ids</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Details regarding the individual's ID documents.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>personal_data.document_ids[].document_type</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The type of document related to the individual. We return one of the following values:
   - `NSS`
@@ -12137,49 +12172,9 @@
 </t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>NSS</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>NSS, CURP, RFC</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>personal_data.document_ids[].document_number</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The ID document's number (as a string).
-</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>10277663582</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -12198,24 +12193,28 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>NSS, CURP, RFC</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>personal_data.email</t>
+          <t>personal_data.document_ids[].document_number</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The email address of the individual.
+          <t xml:space="preserve">The ID document's number (as a string).
 </t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>bruce.banner@avengers.com</t>
+          <t>10277663582</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -12240,63 +12239,59 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>personal_data.email</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The email address of the individual.
+</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>bruce.banner@avengers.com</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>social_security_summary</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Details regarding the individual's social security contributions, according to the IMSS.
 &gt;**Note**: For ISSSTE Mexico, this value will return `null`.
 </t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>object</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>social_security_summary.weeks_redeemed</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Number of weeks the individual needed to take out of their pension.
-</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>int32</t>
-        </is>
-      </c>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -12313,12 +12308,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>social_security_summary.weeks_reinstated</t>
+          <t>social_security_summary.weeks_redeemed</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number of weeks the individual has paid back into their pension (*AFORE*), after having redeemed them previously.
+          <t xml:space="preserve">Number of weeks the individual needed to take out of their pension.
 </t>
         </is>
       </c>
@@ -12353,18 +12348,18 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>social_security_summary.weeks_contributed</t>
+          <t>social_security_summary.weeks_reinstated</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number of weeks the individual has contributed to their social security, based on the number of weeks the individual has worked according to IMSS.
+          <t xml:space="preserve">Number of weeks the individual has paid back into their pension (*AFORE*), after having redeemed them previously.
 </t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -12393,21 +12388,30 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>employment_records</t>
+          <t>social_security_summary.weeks_contributed</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Details regarding the individual's employment history.</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
+          <t xml:space="preserve">Number of weeks the individual has contributed to their social security, based on the number of weeks the individual has worked according to IMSS.
+</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>array</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>int32</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -12415,7 +12419,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -12424,29 +12428,21 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>employment_records[].collected_at</t>
+          <t>employment_records</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>The ISO-8601 timestamp when the data point was collected.</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>2020-04-23T21:32:55.336854+00:00</t>
-        </is>
-      </c>
+          <t>Details regarding the individual's employment history.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>date-time</t>
-        </is>
-      </c>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -12463,104 +12459,103 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>employment_records[].collected_at</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>The ISO-8601 timestamp when the data point was collected.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>2020-04-23T21:32:55.336854+00:00</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>date-time</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>employment_records[].employer</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The official name of the employer.
 &gt;**Note**: For ISSSTE Mexico, this is the official name of the entity along with the entity that is responsible for managing the employee's information, separated by a semicolon (`;`). For example: SECRETARIA DE EDUCACION PUBLICA (SEP);SECRETARIA DE EDUCACION PUBLICA (SEP).
 </t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Batman Enterprises CDMX</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>employment_records[].employer_id</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The official ID of the employer, according to the country.
 &gt;**Note**: For ISSSTE Mexico, this value will return `null`.
 </t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>780-BAT-88769-CDMX</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>employment_records[].start_date</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Date when employment started, in `YYYY-MM-DD` format.
-</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>2019-10-10</t>
-        </is>
-      </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
+      <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -12568,7 +12563,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -12577,71 +12572,71 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>employment_records[].start_date</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date when employment started, in `YYYY-MM-DD` format.
+</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>2019-10-10</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>employment_records[].end_date</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Date when employment finished, in `YYYY-MM-DD` format.
 &gt;**Note**: This field will return `null` for the user's current employment.
 </t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>2019-12-31</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>employment_records[].weeks_employed</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Number of weeks that the individual was employed.
-</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>int32</t>
-        </is>
-      </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -12649,7 +12644,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -12658,47 +12653,87 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t>employment_records[].weeks_employed</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number of weeks that the individual was employed.
+</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>int32</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t>employment_records[].state</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">In what geographical state the individual was employed, according to the country.
 &gt;**Note**: For ISSSTE Mexico, this value will return `null`.
 </t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>DISTRITO FEDERAL</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>employment_records[].most_recent_base_salary</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The most recent base salary the individual earned.
 - For IMSS Mexico, this value is calculated including the perks that the individual is entitled to throughout the year.
@@ -12706,41 +12741,41 @@
 </t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>762.54</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>employment_records[].monthly_salary</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The monthly salary of the individual, including any additional perks.
 - For IMSS Mexico, this value is calculated including the perks that the individual is entitled to throughout the year.
@@ -12748,57 +12783,21 @@
 </t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>23193.925</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>employment_records[].currency</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The three-letter currency code in which the salary is paid.
-</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>MXN</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
           <t>No</t>
@@ -12815,18 +12814,23 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>employment_records[].employment_status_updates</t>
+          <t>employment_records[].currency</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Details regarding any employment changes of the individual.</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr"/>
+          <t xml:space="preserve">The three-letter currency code in which the salary is paid.
+</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -12837,7 +12841,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -12846,10 +12850,41 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>employment_records[].employment_status_updates</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Details regarding any employment changes of the individual.</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
           <t>employment_records[].employment_status_updates[].event</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">For IMSS Mexico, this is the event that caused the change in employment status or salary. We return one of the following values:
   - `DISMISSED_RESIGNED`: The employee was either dismissed or resigned.
@@ -12865,41 +12900,41 @@
 </t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>HIRED</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>DISMISSED_RESIGNED, SALARY_MODIFICATION, HIRED, VOLUNTARY_CONTRIBUTION, ABSENCE, SICK_LEAVE, NORMAL, BDUTA_CERTIFICATE, DYE_CERTIFICATE</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>employment_records[].employment_status_updates[].base_salary</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The base salary of the individual, current as of the `update_date`.
   - For IMSS Mexico, this value is calculated including the perks that the individual is entitled to throughout the year.
@@ -12907,59 +12942,19 @@
 </t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>1033.09</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>number</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>float</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>employment_records[].employment_status_updates[].update_date</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The date that the employment event occurred, in `YYYY-MM-DD` format.
-</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>2021-09-01</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>date</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -12978,10 +12973,50 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>employment_records[].employment_status_updates[].update_date</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The date that the employment event occurred, in `YYYY-MM-DD` format.
+</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>2021-09-01</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
           <t>employment_scores</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">An array of `employment_record` scores. Each score provides an insight into employability and income generation potential in a given period.
 &gt; **Note 1**: This field is only available for links created with Mexico's IMSS. For other institutions, this field will return `null`.
@@ -12989,37 +13024,37 @@
 </t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>[{"score": 722, "period": 3, "version": "1.0.0"}, {"score": 612, "period": 6, "version": "1.0.0"}, {"score": 570, "period": 12, "version": "1.0.0"}]</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>array</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>employment_scores[].score</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">A score between 300 and 900 that provides an insight into employability and income generation potential.
 - A low score (closer to 300) could indicate lower predicted employability and income generation potential, suggesting potential challenges in securing employment or achieving higher income levels in the future.
@@ -13028,37 +13063,37 @@
 </t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>612</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>employment_scores[].period</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The number of months (in the future) that the score is calculated for.
 For example, a period of `6` indicates that the score is calculated for the next `6` months.
@@ -13066,49 +13101,14 @@
 </t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>integer</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>employment_scores[].version</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>The version of our employment score model used to perform the calculation.</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>1.0.0</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>
@@ -13128,18 +13128,22 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>files</t>
+          <t>employment_scores[].version</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Additional PDF binary files relating to the individual's employment.</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr"/>
+          <t>The version of our employment score model used to perform the calculation.</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>array</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -13150,7 +13154,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -13159,23 +13163,20 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>files[].type</t>
+          <t>salary_estimation</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The title of the document.
-</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>ReporteSemanasCotizadas_190123</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Provides a modeled estimation of the user's current base salary and employment status. 
+&gt; **Note**: This field is only available for links created with Mexico's IMSS. For other institutions (such as ISSSTE), this field will return `null`.
+</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>object</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
@@ -13186,7 +13187,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -13195,38 +13196,214 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>salary_estimation.employment_status_estimate</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Current employment status estimated using an employment record with a past report date. Returns `"EMPLOYED"` (if the `base_salary_estimate` is greater than 0) or `"UNEMPLOYED"`.</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>EMPLOYED</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>salary_estimation.base_salary_estimate</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Current base salary (daily amount) estimated using an employment record with a past report date.</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>salary_estimation.currency</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>The three-letter currency code (ISO-4217). For example, `"MXN"`.</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>files</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Additional PDF binary files relating to the individual's employment.</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>files[].type</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The title of the document.
+</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>ReporteSemanasCotizadas_190123</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
           <t>files[].value</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The PDF binary of the file (as a string).
 &gt; **Note**: In our sandbox environment, this field will return `null`.
 </t>
         </is>
       </c>
-      <c r="C47" s="2">
+      <c r="C52" s="2">
         <f>PDF_BINARY=</f>
         <v/>
       </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>